<commit_message>
Corregir puntaje de clasificados y agregar semifinales
</commit_message>
<xml_diff>
--- a/docs/kinela_actualizada.xlsx
+++ b/docs/kinela_actualizada.xlsx
@@ -7,7 +7,8 @@
     <sheet name="Partidos" sheetId="3" r:id="rId3"/>
     <sheet name="Detalle_Participantes" sheetId="4" r:id="rId4"/>
     <sheet name="Antecedente_Octavos" sheetId="5" r:id="rId5"/>
-    <sheet name="Metricas" sheetId="6" r:id="rId6"/>
+    <sheet name="Semifinales" sheetId="6" r:id="rId6"/>
+    <sheet name="Metricas" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -65,7 +66,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-12T03:47:59.785Z</t>
+          <t>2026-07-13T15:05:44.194Z</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -265,17 +266,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P006</t>
+          <t>P005</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Diego</t>
+          <t>Jesús</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>92</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -295,7 +296,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -305,12 +306,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>59</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>33</t>
         </is>
       </c>
     </row>
@@ -322,17 +323,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P005</t>
+          <t>P006</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jesús</t>
+          <t>Diego</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>88</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -347,7 +348,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -362,12 +363,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>56</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>32</t>
         </is>
       </c>
     </row>
@@ -379,37 +380,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>P002</t>
+          <t>P011</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gabriela</t>
+          <t>Jorge</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>84</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -424,7 +425,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -436,17 +437,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P016</t>
+          <t>P018</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Anny</t>
+          <t>Alex</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>78</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -456,12 +457,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -476,12 +477,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>49</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -493,22 +494,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P013</t>
+          <t>P016</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Anny</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>76</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -523,7 +524,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -533,12 +534,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>59</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -550,17 +551,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P018</t>
+          <t>P002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>Gabriela</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>75</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -570,17 +571,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -590,12 +591,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>61</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -607,32 +608,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P007</t>
+          <t>P013</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Aldo</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>74</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -647,12 +648,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>35</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>39</t>
         </is>
       </c>
     </row>
@@ -664,27 +665,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P012</t>
+          <t>P010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Manuel</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -694,7 +695,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -704,12 +705,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>39</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -721,17 +722,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P009</t>
+          <t>P007</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Gino</t>
+          <t>Aldo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>67</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -741,12 +742,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -761,12 +762,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>50</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
     </row>
@@ -778,12 +779,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P011</t>
+          <t>P012</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Jorge</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -803,27 +804,27 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>32</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -835,17 +836,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P008</t>
+          <t>P022</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Javier</t>
+          <t>Óscar</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>58</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -855,12 +856,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -875,12 +876,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>32</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>26</t>
         </is>
       </c>
     </row>
@@ -892,12 +893,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P022</t>
+          <t>P017</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Óscar</t>
+          <t>Moisés</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -907,12 +908,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -922,7 +923,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -932,12 +933,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -949,17 +950,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>P009</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fernando</t>
+          <t>Gino</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>56</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -969,7 +970,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -979,7 +980,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -989,12 +990,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>42</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>14</t>
         </is>
       </c>
     </row>
@@ -1006,17 +1007,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>P017</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Moisés</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1026,12 +1027,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1046,12 +1047,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>25</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>26</t>
         </is>
       </c>
     </row>
@@ -1063,52 +1064,52 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>P010</t>
+          <t>P008</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Manuel</t>
+          <t>Javier</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>44</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1120,12 +1121,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>P023</t>
+          <t>P004</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>manu</t>
+          <t>Juan</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1135,12 +1136,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1150,22 +1151,22 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>36</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1177,17 +1178,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>P004</t>
+          <t>P021</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Juan</t>
+          <t>Diana</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1197,12 +1198,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1217,7 +1218,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>25</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1234,17 +1235,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>P021</t>
+          <t>P014</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Diana</t>
+          <t>José Luis</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1254,12 +1255,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1274,7 +1275,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1291,12 +1292,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>P014</t>
+          <t>P015</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>José Luis</t>
+          <t>Marcelo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1348,12 +1349,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>P015</t>
+          <t>P019</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Marcelo</t>
+          <t>Omar</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1392,63 +1393,6 @@
         </is>
       </c>
       <c r="K23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>P019</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Omar</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1571,7 +1515,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1586,12 +1530,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>["Arthur","manu"]</t>
+          <t>["Arthur","Manuel"]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>159</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1582,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1658,7 +1602,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>166</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1654,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1725,7 +1669,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>32</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1716,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1787,12 +1731,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Moisés"]</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2114,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2217,7 +2161,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2922,7 +2866,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -3251,7 +3195,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3298,7 +3242,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3486,7 +3430,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3560,17 +3504,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3580,7 +3524,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3607,17 +3551,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3627,7 +3571,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3654,17 +3598,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Suplementario</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3701,17 +3645,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3748,17 +3692,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3768,7 +3712,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3795,17 +3739,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>España</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3815,7 +3759,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3842,17 +3786,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3889,17 +3833,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sin envio</t>
+          <t>90 minutos</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3909,7 +3853,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4050,7 +3994,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4238,7 +4182,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4802,7 +4746,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4943,7 +4887,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -5037,7 +4981,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -5178,7 +5122,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5930,7 +5874,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -5981,194 +5925,6 @@
         </is>
       </c>
       <c r="I89" t="inlineStr">
-        <is>
-          <t>confirmed</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>manu</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>QF1</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Francia vs Marruecos</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Francia</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>90 minutos</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>confirmed</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>manu</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>QF2</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>España vs Bélgica</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>90 minutos</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>confirmed</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>manu</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>QF3</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Noruega vs Inglaterra</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Noruega</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Suplementario</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>confirmed</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>manu</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>QF4</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Argentina vs Suiza</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Suiza</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>90 minutos</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
@@ -6389,40 +6145,158 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>metrica</t>
+          <t>partido_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>fase</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>puntos</t>
+          <t>fecha_hora_peru</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>equipo_a</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>equipo_b</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fuente</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>estado</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lider actual</t>
+          <t>SF1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Freddy</t>
+          <t>Semifinal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>2026-07-14T14:00:00-05:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Francia</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ESPN</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Programado</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>SF2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Semifinal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-15T14:00:00-05:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Inglaterra</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ESPN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Programado</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>metrica</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>puntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lider actual</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Freddy</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Partido con mas puntos repartidos</t>
         </is>
       </c>
@@ -6433,7 +6307,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>166</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6319,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>